<commit_message>
Edição brasileira completa: extensões pyRevit e grafos Dynamo em português
- extensões RevitApiBook (Furação, Comprimento, Ocupação, Suportes),
  Comprimento, Suportes e StudioTools traduzidas (zip + fontes em extensoes/)
- 9 grafos Dynamo traduzidos; planilha da WBS e janela de exemplo em PT
- scripts com os nomes do Revit em português (Comentários, FURAÇÃO,
  Qtd suportes, WBS_CODIGO...); tabela em NOMES-PT.md
- removidos os arquivos da edição italiana que tinham sobrado

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TfT7cppXXAzmySC985WA6H
</commit_message>
<xml_diff>
--- a/codice/codice-7-3-tabella.xlsx
+++ b/codice/codice-7-3-tabella.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Parametri" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Codici" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Esempio" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Parâmetros" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Códigos" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Exemplo" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -439,7 +439,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Parametro</t>
+          <t>Parâmetro</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -454,17 +454,17 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Legame</t>
+          <t>Vínculo</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Compilato da</t>
+          <t>Preenchido por</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Descrizione</t>
+          <t>Descrição</t>
         </is>
       </c>
     </row>
@@ -476,27 +476,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>spaziale</t>
+          <t>espacial</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Testo</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Istanza</t>
+          <t>Instância</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>costante di progetto</t>
+          <t>constante do projeto</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Il progetto (SNW)</t>
+          <t>O projeto (SNW)</t>
         </is>
       </c>
     </row>
@@ -508,27 +508,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>spaziale</t>
+          <t>espacial</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Testo</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Istanza</t>
+          <t>Instância</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>smart location (livello)</t>
+          <t>smart location (nível)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Il livello (L01, L02, ...)</t>
+          <t>O nível (L01, L02, ...)</t>
         </is>
       </c>
     </row>
@@ -540,27 +540,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>spaziale</t>
+          <t>espacial</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Testo</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Istanza</t>
+          <t>Instância</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>smart location (locale)</t>
+          <t>smart location (ambiente)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Il locale (R101, ...) o EXT</t>
+          <t>O ambiente (R101, ...) ou EXT</t>
         </is>
       </c>
     </row>
@@ -572,27 +572,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>tecnologico</t>
+          <t>tecnológico</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Testo</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Istanza</t>
+          <t>Instância</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>dizionario per categoria</t>
+          <t>dicionário por categoria</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>La disciplina (ELE, MEC)</t>
+          <t>A disciplina (ELE, MEC)</t>
         </is>
       </c>
     </row>
@@ -604,54 +604,54 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tecnologico</t>
+          <t>tecnológico</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Testo</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Istanza</t>
+          <t>Instância</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>dizionario per categoria</t>
+          <t>dicionário por categoria</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>La categoria (CND, PSS, ...)</t>
+          <t>A categoria (CND, PSS, ...)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>WBS_CODICE</t>
+          <t>WBS_CODIGO</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>aggregato</t>
+          <t>agregado</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Testo</t>
+          <t>Texto</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Istanza</t>
+          <t>Instância</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>lo script, al Passo 3</t>
+          <t>o script, no Passo 3</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -688,17 +688,17 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Codice</t>
+          <t>Código</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Descrizione</t>
+          <t>Descrição</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Da dove viene</t>
+          <t>De onde vem</t>
         </is>
       </c>
     </row>
@@ -720,7 +720,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>costante in testa allo script</t>
+          <t>constante no início do script</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>dal nome del livello</t>
+          <t>do nome do nível</t>
         </is>
       </c>
     </row>
@@ -764,7 +764,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>dal nome del livello</t>
+          <t>do nome do nível</t>
         </is>
       </c>
     </row>
@@ -781,12 +781,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Locale 101</t>
+          <t>Ambiente 101</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>dal numero del Room (link ARC)</t>
+          <t>do número do Room (link ARQ)</t>
         </is>
       </c>
     </row>
@@ -803,12 +803,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Esterno / senza locale</t>
+          <t>Externo / sem ambiente</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>nessun Room contiene il punto</t>
+          <t>nenhum Room contém o ponto</t>
         </is>
       </c>
     </row>
@@ -825,12 +825,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Impianti elettrici</t>
+          <t>Instalações elétricas</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>dizionario per categoria</t>
+          <t>dicionário por categoria</t>
         </is>
       </c>
     </row>
@@ -847,12 +847,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Impianti meccanici</t>
+          <t>Instalações mecânicas</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>dizionario per categoria</t>
+          <t>dicionário por categoria</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cavidotti (tratte e raccordi)</t>
+          <t>Eletrodutos (trechos e conexões)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -891,7 +891,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Passerelle portacavi</t>
+          <t>Eletrocalhas</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -913,7 +913,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Quadri e apparecchiature</t>
+          <t>Quadros e equipamentos</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -935,7 +935,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Forza motrice e prese</t>
+          <t>Força e tomadas</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -957,7 +957,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Illuminazione</t>
+          <t>Iluminação</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -979,7 +979,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Dati e rete</t>
+          <t>Dados e rede</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1001,7 +1001,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Rivelazione incendio</t>
+          <t>Detecção de incêndio</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1023,7 +1023,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Canali aria</t>
+          <t>Dutos de ar</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tubazioni</t>
+          <t>Tubulações</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1110,14 +1110,14 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>WBS_CODICE</t>
+          <t>WBS_CODIGO</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Cavidotto sopra il locale 101</t>
+          <t>Eletroduto sobre o ambiente 101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1154,7 +1154,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Passerella nel corridoio 105</t>
+          <t>Eletrocalha no corredor 105</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1191,7 +1191,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Corpo illuminante esterno</t>
+          <t>Luminária externa</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>